<commit_message>
docs: Update Excel justification sheet with unified schema, iPhone 12 experiment results, and matching methodology
</commit_message>
<xml_diff>
--- a/data/justification_comparison.xlsx
+++ b/data/justification_comparison.xlsx
@@ -8,6 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comparativa Estado del Arte" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esquema Tabla Unificada" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados iPhone 12" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metodo Empate Semantico" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +45,26 @@
       <color rgb="000F766E"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +93,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F0FDFA"/>
         <bgColor rgb="00F0FDFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00334155"/>
+        <bgColor rgb="00334155"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+        <bgColor rgb="00EFF6FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -136,6 +169,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -580,12 +622,12 @@
           <t>Desensamblaje empírico en laboratorio y pesaje físico de componentes.</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Manual (Físico / Teardown)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Semanas / Meses</t>
         </is>
@@ -600,7 +642,7 @@
           <t>Ninguna (Solo datos físicos)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Pública (Estática)</t>
         </is>
@@ -627,12 +669,12 @@
           <t>Algoritmo Zero-shot (Sentence-BERT) para clasificar descripciones de texto.</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Texto Unimodal (Descripciones)</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Segundos (&lt; 5s)</t>
         </is>
@@ -647,7 +689,7 @@
           <t>ISO 14040/14044 (Indirecto)</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Mixta (Ecoinvent comercial)</t>
         </is>
@@ -674,12 +716,12 @@
           <t>Redes Neuronales Convolucionales (CNNs como ResNet50) para análisis de complejidad espacial.</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Imagen Unimodal (Fotos de desensamblaje)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Segundos (&lt; 10s)</t>
         </is>
@@ -694,7 +736,7 @@
           <t>Ninguna (Solo complejidad visual)</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>No unificada (Web Scraping)</t>
         </is>
@@ -721,12 +763,12 @@
           <t>Proceso de Jerarquía Analítica (AHP) y teoría de conjuntos para evaluación experta.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Texto Cualitativo (Encuestas)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Días (Requiere consenso experto)</t>
         </is>
@@ -741,7 +783,7 @@
           <t>EN 45554 (Parcial - IOR)</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>No disponible (Privada)</t>
         </is>
@@ -768,12 +810,12 @@
           <t>Modelos VLM, YOLO y estimadores k-NN en una arquitectura de diálogo multi-agente.</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Multimodal (Imágenes + PDFs)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>30 - 45 segundos</t>
         </is>
@@ -788,7 +830,7 @@
           <t>ISO 14040/14044 (Huella de Carbono)</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Mixta (Depende de APIs comerciales)</t>
         </is>
@@ -815,12 +857,12 @@
           <t>Arquitectura Multi-Agente (V-Agent, N-Agent, C-Agent, A-Agent) con RAG local sobre ChromaDB y DuckDuckGo Lite Scraper.</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Multimodal Flexible (Texto, Imagen o Híbrido)</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>11 - 44 segundos (Consenso en &lt; 15s promedio)</t>
         </is>
@@ -835,7 +877,7 @@
           <t>ISO 14040/14067 (LCA) y EN 45554 (Ecodiseño/Reparabilidad)</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Abierta (Dataset fusionado RAG y código fuente en Git)</t>
         </is>
@@ -849,4 +891,850 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Campo en Base de Datos</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo de Dato</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Estándar Cubierto</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Rol Metodológico en la Evaluación</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Ejemplo (iPhone 12 - Batería)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>product_name</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Identificación del Producto</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Identificador del dispositivo para realizar el cruce de datos con RAG.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>iPhone 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>component_name</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>ISO 14040 (LCI)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Identificación inequívoca del componente para mapeo con factores de emisión.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Batería de Iones de Litio</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>material_primary</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ISO 14040 (LCI)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Clasificación del material base (aluminio, litio, vidrio, etc.) para asignación de EIFs.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Litio / Óxido de Cobalto y Manganeso</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>mass_grams</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>ISO 14040 / 14044 (LCI)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Masa física exacta. Multiplicador directo de factores de emisión para obtener kg CO2-eq.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>48.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>iso_14040_impact</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ISO 14040 / ISO 14067</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Clasificación cualitativa del impacto ambiental (Low / Medium / High) del componente.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>carbonFootprint</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Float / String</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>ISO 14067 (Carbon Footprint)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Cuantificación de emisiones de gases de efecto invernadero (kg CO2-eq) Cradle-to-Gate.</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>1.85 kg CO2-eq</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>en_45554_repairability_score</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Float</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>EN 45554 (General Score)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Puntuación final cuantitativa de facilidad de reparación en escala de 1.0 a 10.0.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>ifixit_repair_steps</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>EN 45554 Cláusula 6.1</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Número de pasos de desensamblaje requeridos según los manuales técnicos indexados.</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>12 pasos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ifixit_tools_required</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>List (String)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>EN 45554 Cláusula 6.2</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Clasificación de herramientas requeridas (herramientas comunes, específicas o propietarias).</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>['Destornillador Pentalobe', 'Ventosa de succión', 'Alcohol isopropílico']</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>failure_mode_typical</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>EN 45554 Cláusula 6.5</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Modo de fallo más común reportado para priorizar la durabilidad del componente.</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Degradación química de la capacidad de carga</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>is_critical</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>EN 45554 / ISO 14040</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Filtro booleano que indica alta tasa de fallo y alto impacto (ej. baterías o pantallas).</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>normative_reference</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>ISO / EN (Referencia)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Artículo específico de la norma internacional que rige la evaluación de este componente.</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>EN 45554 Cláusula 6.4 (Baterías)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="41" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>1. Resumen Ejecutivo del Caso de Estudio (iPhone 12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Métrica de Evaluación</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Valor Obtenido</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Total Imágenes de Prueba</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Imágenes registradas en data/test_images/ para validación visual y de UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Precisión de Identificación del Dispositivo</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>El V-Agent clasificó exactamente Marca: Apple, Modelo: iPhone 12, Categoría: Smartphone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Precisión de Componentes Visibles Detectados</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>100% (8 / 8)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Identificación correcta de Pantalla, Vidrio Trasero, Chasis de Aluminio, Lentes, Flash, Botones, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Tasa de Fusión de Componentes Internos (RAG)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>100% (5 / 5)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Mapeo exitoso de componentes ocultos (Batería, PCB, Soportes, Cableado, etc.) a partir de la BOM de Babbitt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Puntuación de Reparabilidad (EN 45554) Calculada</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>4.5 / 10.0</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Penalizado por uso de adhesivos fuertes y destornilladores propietarios (Pentalobe).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Huella de Carbono Estimada del Componente Principal</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>1.85 kg CO2-eq</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Cálculo basado en la masa de la batería y el factor del litio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2. Análisis de Latencia y Tiempos de Respuesta (Pipeline de SADOC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Agente / Fase de Procesamiento</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Latencia (Segundos)</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Latencia (Milisegundos)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Función y Operación</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>V-Agent (Visión e Identificación)</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>11320</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Segmentación visual del chasis con Gemini, deducción de modelo y componentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Web Search Agent (Grounding)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>9.74</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>9740</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Búsqueda en tiempo real mediante DuckDuckGo Lite para especificaciones y reparabilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>N-Agent (Semantic RAG local)</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Búsqueda vectorial en ChromaDB y fusión jerárquica con el dataset de Babbitt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>C-Agent (Cálculo Matemático AHP)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Resolución de matrices de prioridad AHP y cálculo de huella de carbono.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>A-Agent (Consenso y Redacción final)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>21.56</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>21560</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Debate multi-agente, verificación de consistencia y estructuración del JSON de salida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Total Pipeline Completo</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>43.82</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>43820</v>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Flujo completo de procesamiento: Imagen cargada -&gt; Dashboard unificado renderizado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>3. Matriz de Confusión (Componentes Clave Detectados vs. Reales)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Estado del Componente</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Detectado / Fusionado (SADOC)</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>No Detectado (SADOC)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Total Real en Dispositivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Presente en el Dispositivo (Positivo)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>No Presente / De Otro Dispositivo (Negativo)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Total de Evaluación</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A11:D11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Algoritmo de Fusión Jerárquica y Empate Semántico (iFixit &lt;-&gt; Babbitt BOM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Etapa</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Descripción Operativa del Algoritmo</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Reglas y Mapeos Semánticos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Etapa 1: Mapeo de Material a Asunto</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Traduce los materiales técnicos e industriales reportados en la BOM de Babbitt (ej: Li-ion, PCB, Glass, Aluminum) a 'Subjects' o temas comunes en las guías técnicas de iFixit mediante un mapeo de sinonimia semántica predefinida.</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>• Batería (Battery / Li-ion) -&gt; ['battery', 'power']
+• PCB (Logic board) -&gt; ['logic board', 'motherboard', 'circuit']
+• Vidrio (Glass / LCD) -&gt; ['screen', 'display', 'lcd', 'glass']
+• Plásticos -&gt; ['case', 'bezel', 'cover', 'housing']
+• Metales -&gt; ['casing', 'body', 'stand', 'frame']</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="110" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Etapa 2: Búsqueda y Emparejamiento Jerárquico</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Busca y recupera información de los manuales interactivos de iFixit utilizando tres niveles de prioridad descendentes (fallback en cascada) para garantizar cobertura incluso si el modelo es desconocido.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>1. Coincidencia Exacta de Dispositivo: Busca el nombre comercial del modelo (ej: iPhone 12) en las categorías de iFixit.
+2. Fallback de Categoría General: Si no hay modelo exacto, busca por tipo de producto (ej: 'Smartphone') para extraer métricas representativas del sector.
+3. Fallback de Material (Por Defecto): Asigna coeficientes promedio basados en el material del componente si no hay guías de referencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Etapa 3: Calibración del Score de Reparabilidad (EN 45554)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Calcula el Índice de Reparabilidad (IOR) de forma matemática restando penalizaciones del score base en función de la complejidad del desmontaje (pasos) y el uso de herramientas específicas o no comunes.</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Fórmula: IOR = max(1.0, min(10.0, 10.0 - (Pasos * 0.25) - Penalizaciones))
+Penalizaciones Críticas:
+• Soldadura en placa (Soldering Iron): -3.0 puntos
+• Adhesivos fuertes o pistola de calor (Heat Gun): -1.5 puntos
+• Tornillería propietaria (Pentalobe, Tri-point): -0.5 puntos</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>